<commit_message>
Update confidentiality value set URL in FSH profile fdce4f7d1cff02bec6f717e0098764b63bcd07cd
</commit_message>
<xml_diff>
--- a/nr-securitylabel-slicing-123/ig/StructureDefinition-pdsm-simplified-publish.xlsx
+++ b/nr-securitylabel-slicing-123/ig/StructureDefinition-pdsm-simplified-publish.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-17T12:36:17+00:00</t>
+    <t>2026-10-13T07:43:49+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1189,7 +1189,7 @@
     <t>Niveau de confidentialité standard du document (Normal, Restreint, Très restreint, ...). En l'absence d'information de confidentialité disponible, la valeur par défaut à utiliser est N (Normal), conformément à ce qui est déjà pratiqué aujourd'hui pour les documents CDA.</t>
   </si>
   <si>
-    <t>http://terminology.hl7.org/ValueSet/v3-ConfidentialityClassification</t>
+    <t>http://terminology.hl7.org/ValueSet/v3-Confidentiality</t>
   </si>
   <si>
     <t>DocumentReference.securityLabel:visibilityStatus</t>

</xml_diff>